<commit_message>
ingesta: snapshot 2026-08-02 18:31 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-08-02/CORDOBA_AGO26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-08-02/CORDOBA_AGO26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B5783F-4938-4568-98EA-D052DBF2A83F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C29A3D-D4A5-49FC-B8E3-79BEDC435874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
   <sheets>
     <sheet name="ENERO_2026" sheetId="1" r:id="rId1"/>
@@ -7271,7 +7271,14 @@
     <cellStyle name="Total 2" xfId="426" xr:uid="{C3CBD9B1-F70E-4B3B-902E-48998395073B}"/>
     <cellStyle name="Total 2 2" xfId="1460" xr:uid="{BDD6C7C0-28D1-443D-B7F7-D72827AA1D29}"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.1498764000366222"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -9960,7 +9967,7 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="31"/>
                 <c:pt idx="0">
-                  <c:v>-1</c:v>
+                  <c:v>2.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>-1</c:v>
@@ -14733,53 +14740,53 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E15">
-    <cfRule type="cellIs" dxfId="14" priority="699" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="15" priority="699" stopIfTrue="1" operator="between">
       <formula>40</formula>
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="700" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="14" priority="700" stopIfTrue="1" operator="between">
       <formula>500.1</formula>
       <formula>5000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="701" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="13" priority="701" stopIfTrue="1" operator="between">
       <formula>20</formula>
       <formula>39.999</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="703" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="12" priority="703" stopIfTrue="1" operator="between">
       <formula>500.1</formula>
       <formula>50000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E4:E15">
-    <cfRule type="cellIs" dxfId="10" priority="691" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="11" priority="691" stopIfTrue="1" operator="between">
       <formula>20</formula>
       <formula>1000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:AI15">
-    <cfRule type="cellIs" dxfId="9" priority="698" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="10" priority="698" stopIfTrue="1" operator="between">
       <formula>20</formula>
       <formula>39.99</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="702" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="9" priority="702" stopIfTrue="1" operator="between">
       <formula>40</formula>
       <formula>500</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:AI15">
-    <cfRule type="cellIs" dxfId="7" priority="706" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="8" priority="706" stopIfTrue="1" operator="between">
       <formula>500.1</formula>
       <formula>5000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="707" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="7" priority="707" stopIfTrue="1" operator="between">
       <formula>20</formula>
       <formula>39.999</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="708" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="6" priority="708" stopIfTrue="1" operator="between">
       <formula>40</formula>
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="709" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="5" priority="709" stopIfTrue="1" operator="between">
       <formula>500.1</formula>
       <formula>50000</formula>
     </cfRule>
@@ -16435,7 +16442,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:AI15">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThanOrEqual">
       <formula>50</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18038,7 +18045,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:AI15">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThanOrEqual">
       <formula>50</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19763,7 +19770,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:AI15">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThanOrEqual">
       <formula>50</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19919,7 +19926,9 @@
       <c r="D3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="24"/>
+      <c r="E3" s="24">
+        <v>0</v>
+      </c>
       <c r="F3" s="24"/>
       <c r="G3" s="25"/>
       <c r="H3" s="25"/>
@@ -19971,7 +19980,9 @@
       <c r="D4" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="24"/>
+      <c r="E4" s="24">
+        <v>0</v>
+      </c>
       <c r="F4" s="24"/>
       <c r="G4" s="25"/>
       <c r="H4" s="25"/>
@@ -20023,7 +20034,9 @@
       <c r="D5" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="E5" s="24"/>
+      <c r="E5" s="24">
+        <v>1.5</v>
+      </c>
       <c r="F5" s="24"/>
       <c r="G5" s="25"/>
       <c r="H5" s="25"/>
@@ -20056,7 +20069,7 @@
       <c r="AI5" s="34"/>
       <c r="AJ5" s="36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="AK5" s="30">
         <v>40.986206896551728</v>
@@ -20075,7 +20088,9 @@
       <c r="D6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="24"/>
+      <c r="E6" s="24">
+        <v>0</v>
+      </c>
       <c r="F6" s="24"/>
       <c r="G6" s="25"/>
       <c r="H6" s="25"/>
@@ -20231,7 +20246,9 @@
       <c r="D9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="24"/>
+      <c r="E9" s="24">
+        <v>1</v>
+      </c>
       <c r="F9" s="24"/>
       <c r="G9" s="25"/>
       <c r="H9" s="25"/>
@@ -20264,7 +20281,7 @@
       <c r="AI9" s="34"/>
       <c r="AJ9" s="36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK9" s="30">
         <v>65.482758620689651</v>
@@ -20333,7 +20350,9 @@
       <c r="D11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="24"/>
+      <c r="E11" s="24">
+        <v>0</v>
+      </c>
       <c r="F11" s="24"/>
       <c r="G11" s="25"/>
       <c r="H11" s="25"/>
@@ -20437,7 +20456,9 @@
       <c r="D13" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="24"/>
+      <c r="E13" s="24">
+        <v>0</v>
+      </c>
       <c r="F13" s="24"/>
       <c r="G13" s="25"/>
       <c r="H13" s="25"/>
@@ -20487,7 +20508,9 @@
       <c r="D14" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="24"/>
+      <c r="E14" s="24">
+        <v>0</v>
+      </c>
       <c r="F14" s="24"/>
       <c r="G14" s="25"/>
       <c r="H14" s="25"/>
@@ -20682,7 +20705,7 @@
       </c>
       <c r="E19" s="26">
         <f>IF(COUNT(E3:E17)&gt;0,SUM(E3:E17),-1)</f>
-        <v>-1</v>
+        <v>2.5</v>
       </c>
       <c r="F19" s="26">
         <f t="shared" ref="F19:AI19" si="1">IF(COUNT(F3:F17)&gt;0,SUM(F3:F17),-1)</f>
@@ -20807,7 +20830,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:AI15">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThanOrEqual">
       <formula>50</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>